<commit_message>
updated the Transaction to Rev JE
</commit_message>
<xml_diff>
--- a/Updated Version/Invoice to Rev JE/Journal GL Impacts.xlsx
+++ b/Updated Version/Invoice to Rev JE/Journal GL Impacts.xlsx
@@ -1,19 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorgft1337197-my.sharepoint.com/personal/vishalsurya_arul_zenardy_com/Documents/Vishal Surya/Projects/Netsuite/Kline and Specter/Script/Updated Version/Invoice to Rev JE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="8_{D31E65F5-AE2B-4506-946C-A4BB247A0741}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A5BC726-25DC-49F1-ABE9-32157C70DCA0}"/>
+  <xr:revisionPtr revIDLastSave="148" documentId="8_{D31E65F5-AE2B-4506-946C-A4BB247A0741}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7721F422-0349-47BD-B69E-0DEB1F4812F9}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BC8E91AC-D9CB-4AB0-9262-523B87632849}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{BC8E91AC-D9CB-4AB0-9262-523B87632849}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Final Valdiation" sheetId="4" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId3"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="44">
   <si>
     <t>Hard Costs</t>
   </si>
@@ -99,13 +102,85 @@
   </si>
   <si>
     <t>Customer Payment</t>
+  </si>
+  <si>
+    <t>Transaction Type</t>
+  </si>
+  <si>
+    <t>Matched Transaction Link</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Journal Link</t>
+  </si>
+  <si>
+    <t>https://3594693-sb1.app.netsuite.com/app/accounting/transactions/vendbill.nl?id=48859&amp;whence=&amp;cmid=1779267604069_2049</t>
+  </si>
+  <si>
+    <t>https://3594693-sb1.app.netsuite.com/app/accounting/transactions/journal.nl?id=48860&amp;whence=</t>
+  </si>
+  <si>
+    <t>Expected Result with Matching Acocunts</t>
+  </si>
+  <si>
+    <t>Expected Result with Mismatching Accounts</t>
+  </si>
+  <si>
+    <t>https://3594693-sb1.app.netsuite.com/app/accounting/transactions/custinvc.nl?id=48870&amp;whence=&amp;cmid=1779279243921_2780</t>
+  </si>
+  <si>
+    <t>https://3594693-sb1.app.netsuite.com/app/accounting/transactions/journal.nl?id=48871&amp;whence=</t>
+  </si>
+  <si>
+    <t>https://3594693-sb1.app.netsuite.com/app/accounting/transactions/custpymt.nl?id=48872&amp;whence=&amp;cmid=1779279982005_2833</t>
+  </si>
+  <si>
+    <t>https://3594693-sb1.app.netsuite.com/app/accounting/transactions/journal.nl?id=48873&amp;whence=</t>
+  </si>
+  <si>
+    <t>https://3594693-sb1.app.netsuite.com/app/accounting/transactions/vendpymt.nl?id=48874&amp;whence=&amp;cmid=1779280775329_2910</t>
+  </si>
+  <si>
+    <t>https://3594693-sb1.app.netsuite.com/app/accounting/transactions/journal.nl?id=48875&amp;whence=</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>Reverse JE Created</t>
+  </si>
+  <si>
+    <t>https://3594693-sb1.app.netsuite.com/app/accounting/transactions/vendbill.nl?id=49077&amp;whence=&amp;cmid=1780915792780_660</t>
+  </si>
+  <si>
+    <t>https://3594693-sb1.app.netsuite.com/app/accounting/transactions/journal.nl?id=49078&amp;whence=</t>
+  </si>
+  <si>
+    <t>https://3594693-sb1.app.netsuite.com/app/accounting/transactions/vendpymt.nl?id=49079&amp;whence=&amp;cmid=1780918144901_842</t>
+  </si>
+  <si>
+    <t>https://3594693-sb1.app.netsuite.com/app/accounting/transactions/journal.nl?id=49080&amp;whence=</t>
+  </si>
+  <si>
+    <t>https://3594693-sb1.app.netsuite.com/app/accounting/transactions/custinvc.nl?id=49081&amp;whence=&amp;cmid=1780919114108_955</t>
+  </si>
+  <si>
+    <t>https://3594693-sb1.app.netsuite.com/app/accounting/transactions/journal.nl?id=49082&amp;whence=</t>
+  </si>
+  <si>
+    <t>https://3594693-sb1.app.netsuite.com/app/accounting/transactions/custpymt.nl?id=49083&amp;whence=&amp;cmid=1780919361121_1022</t>
+  </si>
+  <si>
+    <t>https://3594693-sb1.app.netsuite.com/app/accounting/transactions/journal.nl?id=49084&amp;whence=</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -121,8 +196,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -159,8 +242,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -168,14 +257,48 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -188,8 +311,21 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -660,17 +796,17 @@
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="G13" s="4" t="s">
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="G13" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="10"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
@@ -762,12 +898,12 @@
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A23" s="5" t="s">
+      <c r="A23" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="B23" s="5"/>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5"/>
+      <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
@@ -833,12 +969,12 @@
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A32" s="6" t="s">
+      <c r="A32" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B32" s="6"/>
-      <c r="C32" s="6"/>
-      <c r="D32" s="6"/>
+      <c r="B32" s="12"/>
+      <c r="C32" s="12"/>
+      <c r="D32" s="12"/>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B33" t="s">
@@ -906,4 +1042,306 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90772AE3-B9DD-406F-88A6-6A8922AA7F53}">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="41.33203125" style="7" customWidth="1"/>
+    <col min="3" max="3" width="26.6640625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="49.5546875" style="7" customWidth="1"/>
+    <col min="5" max="16384" width="8.88671875" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D1" s="16" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{7EF38129-E3CA-41C5-9471-8646BBF8ED19}"/>
+    <hyperlink ref="D2" r:id="rId2" xr:uid="{8AFA0361-EE18-4C47-AF38-2804350E2DD7}"/>
+    <hyperlink ref="B3" r:id="rId3" xr:uid="{3C169F8A-BCFB-4F57-A039-A5D13391BFFE}"/>
+    <hyperlink ref="D3" r:id="rId4" xr:uid="{F9BEA7B1-7796-41F9-8547-63164FED9089}"/>
+    <hyperlink ref="B4" r:id="rId5" xr:uid="{2B067CC8-C60F-4CC4-823B-F60AB48F0EF2}"/>
+    <hyperlink ref="D4" r:id="rId6" xr:uid="{35CEE325-77DB-4D5C-9BC3-8067F8BCA067}"/>
+    <hyperlink ref="B5" r:id="rId7" xr:uid="{C3377C0A-542B-4730-9F17-6DEF581E7537}"/>
+    <hyperlink ref="D5" r:id="rId8" xr:uid="{97116EC8-2D87-427F-95C8-F7866866BC42}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId9"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82B38CBC-BD5F-478A-AD51-00C1CA55006D}">
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.44140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="38.44140625" style="7" customWidth="1"/>
+    <col min="5" max="5" width="28.109375" style="7" customWidth="1"/>
+    <col min="6" max="16384" width="8.88671875" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+    </row>
+    <row r="4" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{A5589BF3-1814-4FCA-B09C-C731D85A7B72}"/>
+    <hyperlink ref="E2" r:id="rId2" xr:uid="{F1155C1C-DC0E-4C32-A716-ADA52F95A202}"/>
+    <hyperlink ref="D4" r:id="rId3" xr:uid="{21008AC9-7892-43E4-85EF-95A096665FA4}"/>
+    <hyperlink ref="E4" r:id="rId4" xr:uid="{92025042-545D-4891-8128-7D90393F7CE5}"/>
+    <hyperlink ref="D5" r:id="rId5" xr:uid="{A31B1DF3-9CDF-41A7-A154-BDEA7A628B45}"/>
+    <hyperlink ref="E5" r:id="rId6" xr:uid="{59175405-76FD-48B1-A09B-C639E5C4E9C0}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId7"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D9A4135-3E57-4ED8-8F36-BB634BE0DFA4}">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="18.21875" customWidth="1"/>
+    <col min="2" max="2" width="44.21875" customWidth="1"/>
+    <col min="3" max="3" width="35.77734375" customWidth="1"/>
+    <col min="4" max="4" width="36.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{7A774F05-3BB6-4CF7-80F8-70ADFE0EE6CD}"/>
+    <hyperlink ref="D2" r:id="rId2" xr:uid="{4C04F952-8A47-4A49-9A69-8B9FCDE3EC5E}"/>
+    <hyperlink ref="C4" r:id="rId3" xr:uid="{F0E231BD-8C97-4E21-90CD-5CBB80595382}"/>
+    <hyperlink ref="D4" r:id="rId4" xr:uid="{AAC2305D-6278-4901-BE57-02EDBB456CC0}"/>
+    <hyperlink ref="C5" r:id="rId5" xr:uid="{EE82760C-CE3D-4E87-AB73-8E5321920617}"/>
+    <hyperlink ref="D5" r:id="rId6" xr:uid="{C6C07466-8CFC-4333-AE2B-8E938C146A2F}"/>
+    <hyperlink ref="C3" r:id="rId7" xr:uid="{613655BB-26BE-4C7A-8593-9A5784F55A0A}"/>
+    <hyperlink ref="D3" r:id="rId8" xr:uid="{DB03B147-9558-4FD7-B12F-D72AE12BAC3B}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>